<commit_message>
Excel: map key and value rows, server roles, id references
</commit_message>
<xml_diff>
--- a/tests/fixtures/excel/full-odcs-3.2.xlsx
+++ b/tests/fixtures/excel/full-odcs-3.2.xlsx
@@ -16555,7 +16555,6 @@
     </row>
     <row r="12">
       <c r="A12" s="34" t="n"/>
-      <c r="B12" s="34" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
@@ -16684,7 +16683,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="34" t="inlineStr">
         <is>
@@ -18009,7 +18007,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>
@@ -20205,7 +20202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ52"/>
+  <dimension ref="A1:AZ55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="34.83203125" customWidth="1" style="2" min="1" max="1"/>
@@ -20253,7 +20250,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>
@@ -22166,104 +22162,50 @@
       <c r="AZ34" s="15" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>attributes</t>
-        </is>
-      </c>
-      <c r="B35" s="15" t="inlineStr">
-        <is>
-          <t>Attributes</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="15" t="inlineStr">
-        <is>
-          <t>Free-form key/value attributes.</t>
-        </is>
-      </c>
-      <c r="G35" s="15" t="n"/>
-      <c r="H35" s="15" t="n"/>
-      <c r="I35" s="15" t="inlineStr">
-        <is>
-          <t>internal</t>
-        </is>
-      </c>
-      <c r="J35" s="15" t="n"/>
-      <c r="K35" s="15" t="n"/>
-      <c r="L35" s="15" t="n"/>
-      <c r="M35" s="15" t="n"/>
-      <c r="N35" s="15" t="n"/>
-      <c r="O35" s="15" t="n"/>
-      <c r="P35" s="15" t="n"/>
-      <c r="Q35" s="15" t="n"/>
-      <c r="R35" s="15" t="n"/>
-      <c r="S35" s="15" t="n"/>
-      <c r="T35" s="15" t="n"/>
-      <c r="U35" s="15" t="n"/>
-      <c r="V35" s="15" t="n"/>
-      <c r="W35" s="15" t="n"/>
-      <c r="X35" s="15" t="n"/>
-      <c r="Y35" s="15" t="n"/>
-      <c r="Z35" s="15" t="n"/>
-      <c r="AA35" s="15" t="n"/>
-      <c r="AB35" s="15" t="n"/>
-      <c r="AC35" s="15" t="n"/>
-      <c r="AD35" s="15" t="n"/>
-      <c r="AE35" s="15" t="n"/>
-      <c r="AF35" s="15" t="n"/>
-      <c r="AG35" s="15" t="n"/>
-      <c r="AH35" s="15" t="n"/>
-      <c r="AI35" s="15" t="n"/>
-      <c r="AJ35" s="15" t="n"/>
-      <c r="AK35" s="15" t="n"/>
-      <c r="AL35" s="15" t="n"/>
-      <c r="AM35" s="15" t="n"/>
-      <c r="AV35" s="15" t="inlineStr">
-        <is>
-          <t>shipmentsAttributes</t>
-        </is>
-      </c>
-      <c r="AW35" s="28" t="n"/>
-      <c r="AX35" s="15" t="n"/>
-      <c r="AY35" s="15" t="n"/>
-      <c r="AZ35" s="15" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>handling_tags.items</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="AD35" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>description_embedding</t>
+          <t>attributes</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>Description Embedding</t>
+          <t>Attributes</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>map</t>
         </is>
       </c>
       <c r="E36" s="16" t="n"/>
       <c r="F36" s="15" t="inlineStr">
         <is>
-          <t>Embedding of the shipment description.</t>
+          <t>Free-form key/value attributes.</t>
         </is>
       </c>
       <c r="G36" s="15" t="n"/>
@@ -22303,35 +22245,9 @@
       <c r="AK36" s="15" t="n"/>
       <c r="AL36" s="15" t="n"/>
       <c r="AM36" s="15" t="n"/>
-      <c r="AN36" t="n">
-        <v>1536</v>
-      </c>
-      <c r="AO36" t="inlineStr">
-        <is>
-          <t>float32</t>
-        </is>
-      </c>
-      <c r="AP36" t="inlineStr">
-        <is>
-          <t>cosine</t>
-        </is>
-      </c>
-      <c r="AQ36" t="b">
-        <v>1</v>
-      </c>
-      <c r="AR36" t="inlineStr">
-        <is>
-          <t>text-embedding-3-small</t>
-        </is>
-      </c>
-      <c r="AS36" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AV36" s="15" t="inlineStr">
         <is>
-          <t>shipmentsEmbedding</t>
+          <t>shipmentsAttributes</t>
         </is>
       </c>
       <c r="AW36" s="28" t="n"/>
@@ -22340,135 +22256,73 @@
       <c r="AZ36" s="15" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>delivery_note</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="inlineStr">
-        <is>
-          <t>Delivery Note</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>attributes.key</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="15" t="inlineStr">
-        <is>
-          <t>Free-text note captured at handover.</t>
-        </is>
-      </c>
-      <c r="G37" s="15" t="n"/>
-      <c r="H37" s="15" t="n"/>
-      <c r="I37" s="15" t="inlineStr">
-        <is>
-          <t>restricted</t>
-        </is>
-      </c>
-      <c r="J37" s="15" t="n"/>
-      <c r="K37" s="15" t="n"/>
-      <c r="L37" s="15" t="n"/>
-      <c r="M37" s="15" t="n"/>
-      <c r="N37" s="15" t="n"/>
-      <c r="O37" s="15" t="n"/>
-      <c r="P37" s="15" t="n"/>
-      <c r="Q37" s="15" t="n"/>
-      <c r="R37" s="15" t="n"/>
-      <c r="S37" s="15" t="n"/>
-      <c r="T37" s="15" t="n"/>
-      <c r="U37" s="15" t="n"/>
-      <c r="V37" s="15" t="n"/>
-      <c r="W37" s="15" t="n"/>
-      <c r="X37" s="15" t="n"/>
-      <c r="Y37" s="15" t="n"/>
-      <c r="Z37" s="15" t="n"/>
-      <c r="AA37" s="15" t="n"/>
-      <c r="AB37" s="15" t="n"/>
-      <c r="AC37" s="15" t="n"/>
-      <c r="AD37" s="15" t="n"/>
-      <c r="AE37" s="15" t="n"/>
-      <c r="AF37" s="15" t="n"/>
-      <c r="AG37" s="15" t="n"/>
-      <c r="AH37" s="15" t="n"/>
-      <c r="AI37" s="15" t="n"/>
-      <c r="AJ37" s="15" t="n"/>
-      <c r="AK37" s="15" t="n"/>
-      <c r="AL37" s="15" t="n"/>
-      <c r="AM37" s="15" t="n"/>
-      <c r="AV37" s="15" t="inlineStr">
-        <is>
-          <t>shipmentsDeliveryNote</t>
-        </is>
-      </c>
-      <c r="AW37" s="28" t="n"/>
-      <c r="AX37" s="15" t="n"/>
-      <c r="AY37" s="15" t="n"/>
-      <c r="AZ37" s="15" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="n"/>
-      <c r="B38" s="15" t="n"/>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="15" t="n"/>
-      <c r="H38" s="15" t="n"/>
-      <c r="I38" s="15" t="n"/>
-      <c r="J38" s="15" t="n"/>
-      <c r="K38" s="15" t="n"/>
-      <c r="L38" s="15" t="n"/>
-      <c r="M38" s="15" t="n"/>
-      <c r="N38" s="15" t="n"/>
-      <c r="O38" s="15" t="n"/>
-      <c r="P38" s="15" t="n"/>
-      <c r="Q38" s="15" t="n"/>
-      <c r="R38" s="15" t="n"/>
-      <c r="S38" s="15" t="n"/>
-      <c r="T38" s="15" t="n"/>
-      <c r="U38" s="15" t="n"/>
-      <c r="V38" s="15" t="n"/>
-      <c r="W38" s="15" t="n"/>
-      <c r="X38" s="15" t="n"/>
-      <c r="Y38" s="15" t="n"/>
-      <c r="Z38" s="15" t="n"/>
-      <c r="AA38" s="15" t="n"/>
-      <c r="AB38" s="15" t="n"/>
-      <c r="AC38" s="15" t="n"/>
-      <c r="AD38" s="15" t="n"/>
-      <c r="AE38" s="15" t="n"/>
-      <c r="AF38" s="15" t="n"/>
-      <c r="AG38" s="15" t="n"/>
-      <c r="AH38" s="15" t="n"/>
-      <c r="AI38" s="15" t="n"/>
-      <c r="AJ38" s="15" t="n"/>
-      <c r="AK38" s="15" t="n"/>
-      <c r="AL38" s="15" t="n"/>
-      <c r="AM38" s="15" t="n"/>
-      <c r="AV38" s="15" t="n"/>
-      <c r="AW38" s="28" t="n"/>
-      <c r="AX38" s="15" t="n"/>
-      <c r="AY38" s="15" t="n"/>
-      <c r="AZ38" s="15" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>attributes.value</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="n"/>
-      <c r="B39" s="15" t="n"/>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>description_embedding</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>Description Embedding</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
       <c r="E39" s="16" t="n"/>
-      <c r="F39" s="15" t="n"/>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>Embedding of the shipment description.</t>
+        </is>
+      </c>
       <c r="G39" s="15" t="n"/>
       <c r="H39" s="15" t="n"/>
-      <c r="I39" s="15" t="n"/>
+      <c r="I39" s="15" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
       <c r="J39" s="15" t="n"/>
       <c r="K39" s="15" t="n"/>
       <c r="L39" s="15" t="n"/>
@@ -22499,22 +22353,76 @@
       <c r="AK39" s="15" t="n"/>
       <c r="AL39" s="15" t="n"/>
       <c r="AM39" s="15" t="n"/>
-      <c r="AV39" s="15" t="n"/>
+      <c r="AN39" t="n">
+        <v>1536</v>
+      </c>
+      <c r="AO39" t="inlineStr">
+        <is>
+          <t>float32</t>
+        </is>
+      </c>
+      <c r="AP39" t="inlineStr">
+        <is>
+          <t>cosine</t>
+        </is>
+      </c>
+      <c r="AQ39" t="b">
+        <v>1</v>
+      </c>
+      <c r="AR39" t="inlineStr">
+        <is>
+          <t>text-embedding-3-small</t>
+        </is>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AV39" s="15" t="inlineStr">
+        <is>
+          <t>shipmentsEmbedding</t>
+        </is>
+      </c>
       <c r="AW39" s="28" t="n"/>
       <c r="AX39" s="15" t="n"/>
       <c r="AY39" s="15" t="n"/>
       <c r="AZ39" s="15" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="n"/>
-      <c r="B40" s="15" t="n"/>
-      <c r="C40" s="15" t="n"/>
-      <c r="D40" s="15" t="n"/>
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>delivery_note</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>Delivery Note</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
       <c r="E40" s="16" t="n"/>
-      <c r="F40" s="15" t="n"/>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>Free-text note captured at handover.</t>
+        </is>
+      </c>
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="15" t="n"/>
-      <c r="I40" s="15" t="n"/>
+      <c r="I40" s="15" t="inlineStr">
+        <is>
+          <t>restricted</t>
+        </is>
+      </c>
       <c r="J40" s="15" t="n"/>
       <c r="K40" s="15" t="n"/>
       <c r="L40" s="15" t="n"/>
@@ -22545,7 +22453,11 @@
       <c r="AK40" s="15" t="n"/>
       <c r="AL40" s="15" t="n"/>
       <c r="AM40" s="15" t="n"/>
-      <c r="AV40" s="15" t="n"/>
+      <c r="AV40" s="15" t="inlineStr">
+        <is>
+          <t>shipmentsDeliveryNote</t>
+        </is>
+      </c>
       <c r="AW40" s="28" t="n"/>
       <c r="AX40" s="15" t="n"/>
       <c r="AY40" s="15" t="n"/>
@@ -23102,6 +23014,144 @@
       <c r="AX52" s="15" t="n"/>
       <c r="AY52" s="15" t="n"/>
       <c r="AZ52" s="15" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="15" t="n"/>
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="16" t="n"/>
+      <c r="F53" s="15" t="n"/>
+      <c r="G53" s="15" t="n"/>
+      <c r="H53" s="15" t="n"/>
+      <c r="I53" s="15" t="n"/>
+      <c r="J53" s="15" t="n"/>
+      <c r="K53" s="15" t="n"/>
+      <c r="L53" s="15" t="n"/>
+      <c r="M53" s="15" t="n"/>
+      <c r="N53" s="15" t="n"/>
+      <c r="O53" s="15" t="n"/>
+      <c r="P53" s="15" t="n"/>
+      <c r="Q53" s="15" t="n"/>
+      <c r="R53" s="15" t="n"/>
+      <c r="S53" s="15" t="n"/>
+      <c r="T53" s="15" t="n"/>
+      <c r="U53" s="15" t="n"/>
+      <c r="V53" s="15" t="n"/>
+      <c r="W53" s="15" t="n"/>
+      <c r="X53" s="15" t="n"/>
+      <c r="Y53" s="15" t="n"/>
+      <c r="Z53" s="15" t="n"/>
+      <c r="AA53" s="15" t="n"/>
+      <c r="AB53" s="15" t="n"/>
+      <c r="AC53" s="15" t="n"/>
+      <c r="AD53" s="15" t="n"/>
+      <c r="AE53" s="15" t="n"/>
+      <c r="AF53" s="15" t="n"/>
+      <c r="AG53" s="15" t="n"/>
+      <c r="AH53" s="15" t="n"/>
+      <c r="AI53" s="15" t="n"/>
+      <c r="AJ53" s="15" t="n"/>
+      <c r="AK53" s="15" t="n"/>
+      <c r="AL53" s="15" t="n"/>
+      <c r="AM53" s="15" t="n"/>
+      <c r="AV53" s="15" t="n"/>
+      <c r="AW53" s="28" t="n"/>
+      <c r="AX53" s="15" t="n"/>
+      <c r="AY53" s="15" t="n"/>
+      <c r="AZ53" s="15" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="15" t="n"/>
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="16" t="n"/>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="15" t="n"/>
+      <c r="H54" s="15" t="n"/>
+      <c r="I54" s="15" t="n"/>
+      <c r="J54" s="15" t="n"/>
+      <c r="K54" s="15" t="n"/>
+      <c r="L54" s="15" t="n"/>
+      <c r="M54" s="15" t="n"/>
+      <c r="N54" s="15" t="n"/>
+      <c r="O54" s="15" t="n"/>
+      <c r="P54" s="15" t="n"/>
+      <c r="Q54" s="15" t="n"/>
+      <c r="R54" s="15" t="n"/>
+      <c r="S54" s="15" t="n"/>
+      <c r="T54" s="15" t="n"/>
+      <c r="U54" s="15" t="n"/>
+      <c r="V54" s="15" t="n"/>
+      <c r="W54" s="15" t="n"/>
+      <c r="X54" s="15" t="n"/>
+      <c r="Y54" s="15" t="n"/>
+      <c r="Z54" s="15" t="n"/>
+      <c r="AA54" s="15" t="n"/>
+      <c r="AB54" s="15" t="n"/>
+      <c r="AC54" s="15" t="n"/>
+      <c r="AD54" s="15" t="n"/>
+      <c r="AE54" s="15" t="n"/>
+      <c r="AF54" s="15" t="n"/>
+      <c r="AG54" s="15" t="n"/>
+      <c r="AH54" s="15" t="n"/>
+      <c r="AI54" s="15" t="n"/>
+      <c r="AJ54" s="15" t="n"/>
+      <c r="AK54" s="15" t="n"/>
+      <c r="AL54" s="15" t="n"/>
+      <c r="AM54" s="15" t="n"/>
+      <c r="AV54" s="15" t="n"/>
+      <c r="AW54" s="28" t="n"/>
+      <c r="AX54" s="15" t="n"/>
+      <c r="AY54" s="15" t="n"/>
+      <c r="AZ54" s="15" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="15" t="n"/>
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="16" t="n"/>
+      <c r="F55" s="15" t="n"/>
+      <c r="G55" s="15" t="n"/>
+      <c r="H55" s="15" t="n"/>
+      <c r="I55" s="15" t="n"/>
+      <c r="J55" s="15" t="n"/>
+      <c r="K55" s="15" t="n"/>
+      <c r="L55" s="15" t="n"/>
+      <c r="M55" s="15" t="n"/>
+      <c r="N55" s="15" t="n"/>
+      <c r="O55" s="15" t="n"/>
+      <c r="P55" s="15" t="n"/>
+      <c r="Q55" s="15" t="n"/>
+      <c r="R55" s="15" t="n"/>
+      <c r="S55" s="15" t="n"/>
+      <c r="T55" s="15" t="n"/>
+      <c r="U55" s="15" t="n"/>
+      <c r="V55" s="15" t="n"/>
+      <c r="W55" s="15" t="n"/>
+      <c r="X55" s="15" t="n"/>
+      <c r="Y55" s="15" t="n"/>
+      <c r="Z55" s="15" t="n"/>
+      <c r="AA55" s="15" t="n"/>
+      <c r="AB55" s="15" t="n"/>
+      <c r="AC55" s="15" t="n"/>
+      <c r="AD55" s="15" t="n"/>
+      <c r="AE55" s="15" t="n"/>
+      <c r="AF55" s="15" t="n"/>
+      <c r="AG55" s="15" t="n"/>
+      <c r="AH55" s="15" t="n"/>
+      <c r="AI55" s="15" t="n"/>
+      <c r="AJ55" s="15" t="n"/>
+      <c r="AK55" s="15" t="n"/>
+      <c r="AL55" s="15" t="n"/>
+      <c r="AM55" s="15" t="n"/>
+      <c r="AV55" s="15" t="n"/>
+      <c r="AW55" s="28" t="n"/>
+      <c r="AX55" s="15" t="n"/>
+      <c r="AY55" s="15" t="n"/>
+      <c r="AZ55" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -23209,7 +23259,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel: vendor the published template and conformance pair
</commit_message>
<xml_diff>
--- a/tests/fixtures/excel/full-odcs-3.2.xlsx
+++ b/tests/fixtures/excel/full-odcs-3.2.xlsx
@@ -35,7 +35,7 @@
     <definedName name="authoritativeDefinitions">'Authoritative Definitions'!$A$4:$F$1000</definedName>
     <definedName name="constraints">Constraints!$A$4:$AZ$1000</definedName>
     <definedName name="context.instructions">Fundamentals!$C$26</definedName>
-    <definedName name="CustomProperties">'Custom Properties'!$A$5:$G$21</definedName>
+    <definedName name="CustomProperties">'Custom Properties'!$A$5:$H$21</definedName>
     <definedName name="datacontract_id">Fundamentals!$C$7</definedName>
     <definedName name="dataProduct">Fundamentals!$C$16</definedName>
     <definedName name="description.limitations">Fundamentals!$C$21</definedName>
@@ -87,7 +87,7 @@
     <definedName name="support">Support!$A$4:$AZ$1000</definedName>
     <definedName name="synonyms">Synonyms!$A$4:$AZ$1000</definedName>
     <definedName name="tags">Fundamentals!$C$24</definedName>
-    <definedName name="team">Team!$A$10:$AZ$1006</definedName>
+    <definedName name="team">Team!$A$10:$BA$1006</definedName>
     <definedName name="team.description">Team!$B$5</definedName>
     <definedName name="team.id">Team!$B$7</definedName>
     <definedName name="team.name">Team!$B$4</definedName>

</xml_diff>